<commit_message>
Add contract price disclaimer
</commit_message>
<xml_diff>
--- a/assets/files/quotes/ABADI-quotation.xlsx
+++ b/assets/files/quotes/ABADI-quotation.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -524,7 +524,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>人民币（RMB）参考价；最终以双方确认采购清单为准</t>
+          <t>人民币（RMB）参考价；最终价格以双方签署的合同价格为准</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr"/>
@@ -1235,6 +1235,20 @@
       </c>
       <c r="C43" s="2" t="inlineStr"/>
       <c r="D43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44" ht="24" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>报价说明</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>页面与本表报价均为参考资料，最终价格以双方签署的合同价格为准。</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>